<commit_message>
Mark 5 kaomoji faces as player-verified
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kaomoji_Alt_Emporium_Tracker.xlsx
+++ b/Kaomoji_Alt_Emporium_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tucke\AppData\Local\Temp\claude\C--Users-tucke-Github-tuckermills-portfolio\33b1b9ce-b7db-4dbc-9e1e-2990ef1ad3b2\scratchpad\xlsx-build\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tucke\Github\ffxi-kaomoji\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D9326DF-8E52-41DF-A42A-645EFC92AC3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FD71B6-579B-4D09-9F0F-7E36AA3E105C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="4290" windowWidth="38700" windowHeight="15885" xr2:uid="{2D23F0FE-9A19-4136-B62C-F2C850B745CA}"/>
+    <workbookView xWindow="17230" yWindow="14400" windowWidth="19380" windowHeight="21690" xr2:uid="{2D23F0FE-9A19-4136-B62C-F2C850B745CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Entries" sheetId="1" r:id="rId1"/>
@@ -1809,7 +1809,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
@@ -1820,7 +1820,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
@@ -1831,7 +1831,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
@@ -1842,7 +1842,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">
@@ -1853,7 +1853,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16.5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update site with latest FFXI testing results
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kaomoji_Alt_Emporium_Tracker.xlsx
+++ b/Kaomoji_Alt_Emporium_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tucke\Github\ffxi-kaomoji\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{890F6205-D70E-43E0-8B17-4E8EAD536516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F31B351-D199-4FCF-9CB0-452B5A2FF66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="38700" windowHeight="15885" xr2:uid="{0B1086ED-8FCA-485A-865A-06293B9ADB03}"/>
+    <workbookView xWindow="-1970" yWindow="14400" windowWidth="19380" windowHeight="21690" xr2:uid="{0B1086ED-8FCA-485A-865A-06293B9ADB03}"/>
   </bookViews>
   <sheets>
     <sheet name="Entries" sheetId="1" r:id="rId1"/>
@@ -3555,7 +3555,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>17</v>
@@ -3575,7 +3575,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>17</v>
@@ -3595,7 +3595,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>22</v>
@@ -3615,7 +3615,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>22</v>
@@ -3635,7 +3635,7 @@
         <v>9</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>22</v>

</xml_diff>

<commit_message>
Sync latest testing statuses
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kaomoji_Alt_Emporium_Tracker.xlsx
+++ b/Kaomoji_Alt_Emporium_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tucke\Github\ffxi-kaomoji\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD248598-690E-4691-975B-D2BAE96FFE9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6401A95-B476-4AB8-878D-87A98D0FF194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="2730" windowWidth="38700" windowHeight="15885" xr2:uid="{0B1086ED-8FCA-485A-865A-06293B9ADB03}"/>
   </bookViews>
@@ -4396,7 +4396,7 @@
         <v>9</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
@@ -4410,7 +4410,7 @@
         <v>9</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
@@ -4424,7 +4424,7 @@
         <v>9</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="5"/>

</xml_diff>

<commit_message>
Add 48 building blocks extracted from existing kaomoji faces
Every non-ASCII character used across the 54 kaomoji faces that wasn't
already a standalone Kaomoji Part, so individual characters from an
unsupported face (which may not be the reason it failed) can be tested
on their own. Left as Untested for manual verification in-game.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kaomoji_Alt_Emporium_Tracker.xlsx
+++ b/Kaomoji_Alt_Emporium_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tucke\Github\ffxi-kaomoji\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6401A95-B476-4AB8-878D-87A98D0FF194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD5EBEC-E534-4A2D-84D7-792D476D5461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2730" yWindow="2730" windowWidth="38700" windowHeight="15885" xr2:uid="{0B1086ED-8FCA-485A-865A-06293B9ADB03}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Entries!$A$4:$F$434</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Entries!$A$4:$F$482</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2575" uniqueCount="976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2767" uniqueCount="1063">
   <si>
     <t>Kaomoji Alt Emporium — Content Database</t>
   </si>
@@ -2982,6 +2982,267 @@
   </si>
   <si>
     <t xml:space="preserve">(つ☆ω☆)つ </t>
+  </si>
+  <si>
+    <t>́</t>
+  </si>
+  <si>
+    <t>Combining acute accent</t>
+  </si>
+  <si>
+    <t>̀</t>
+  </si>
+  <si>
+    <t>Combining grave accent</t>
+  </si>
+  <si>
+    <t>︵</t>
+  </si>
+  <si>
+    <t>Vertical left parenthesis (table-flip arm)</t>
+  </si>
+  <si>
+    <t>｡</t>
+  </si>
+  <si>
+    <t>Halfwidth ideographic full stop</t>
+  </si>
+  <si>
+    <t>／</t>
+  </si>
+  <si>
+    <t>Fullwidth slash</t>
+  </si>
+  <si>
+    <t>；</t>
+  </si>
+  <si>
+    <t>Fullwidth semicolon</t>
+  </si>
+  <si>
+    <t>＠</t>
+  </si>
+  <si>
+    <t>Fullwidth at sign</t>
+  </si>
+  <si>
+    <t>＼</t>
+  </si>
+  <si>
+    <t>Fullwidth backslash</t>
+  </si>
+  <si>
+    <t>﹏</t>
+  </si>
+  <si>
+    <t>Wavy low line</t>
+  </si>
+  <si>
+    <t>｀</t>
+  </si>
+  <si>
+    <t>Fullwidth grave accent</t>
+  </si>
+  <si>
+    <t>～</t>
+  </si>
+  <si>
+    <t>Fullwidth tilde</t>
+  </si>
+  <si>
+    <t>￣</t>
+  </si>
+  <si>
+    <t>Fullwidth macron</t>
+  </si>
+  <si>
+    <t>‿</t>
+  </si>
+  <si>
+    <t>Undertie (smile mouth)</t>
+  </si>
+  <si>
+    <t>︿</t>
+  </si>
+  <si>
+    <t>Vertical caret (frown mouth)</t>
+  </si>
+  <si>
+    <t>∀</t>
+  </si>
+  <si>
+    <t>For-all sign</t>
+  </si>
+  <si>
+    <t>∇</t>
+  </si>
+  <si>
+    <t>Nabla</t>
+  </si>
+  <si>
+    <t>⊂</t>
+  </si>
+  <si>
+    <t>Subset sign (arm)</t>
+  </si>
+  <si>
+    <t>⊃</t>
+  </si>
+  <si>
+    <t>Superset sign (arm)</t>
+  </si>
+  <si>
+    <t>◕</t>
+  </si>
+  <si>
+    <t>Circle, lower-right half black (eye)</t>
+  </si>
+  <si>
+    <t>◡</t>
+  </si>
+  <si>
+    <t>Lower half circle (smile mouth)</t>
+  </si>
+  <si>
+    <t>━</t>
+  </si>
+  <si>
+    <t>Heavy horizontal line</t>
+  </si>
+  <si>
+    <t>Box corner, up+right</t>
+  </si>
+  <si>
+    <t>Box corner, up+left</t>
+  </si>
+  <si>
+    <t>╯</t>
+  </si>
+  <si>
+    <t>Rounded corner, up+left (table-flip arm)</t>
+  </si>
+  <si>
+    <t>┻</t>
+  </si>
+  <si>
+    <t>Heavy T-junction (table)</t>
+  </si>
+  <si>
+    <t>Double cross junction</t>
+  </si>
+  <si>
+    <t>・</t>
+  </si>
+  <si>
+    <t>Katakana middle dot</t>
+  </si>
+  <si>
+    <t>☆</t>
+  </si>
+  <si>
+    <t>White star</t>
+  </si>
+  <si>
+    <t>♡</t>
+  </si>
+  <si>
+    <t>White heart</t>
+  </si>
+  <si>
+    <t>๑</t>
+  </si>
+  <si>
+    <t>Thai digit one (decorative)</t>
+  </si>
+  <si>
+    <t>۶</t>
+  </si>
+  <si>
+    <t>Arabic-indic digit six (decorative arm)</t>
+  </si>
+  <si>
+    <t>٩</t>
+  </si>
+  <si>
+    <t>Arabic-indic digit nine (decorative arm)</t>
+  </si>
+  <si>
+    <t>ｏ</t>
+  </si>
+  <si>
+    <t>Fullwidth letter o</t>
+  </si>
+  <si>
+    <t>ｗ</t>
+  </si>
+  <si>
+    <t>Fullwidth letter w</t>
+  </si>
+  <si>
+    <t>っ</t>
+  </si>
+  <si>
+    <t>Hiragana small tsu</t>
+  </si>
+  <si>
+    <t>ツ</t>
+  </si>
+  <si>
+    <t>Katakana tsu (shrug face)</t>
+  </si>
+  <si>
+    <t>つ</t>
+  </si>
+  <si>
+    <t>Hiragana tsu (arm)</t>
+  </si>
+  <si>
+    <t>づ</t>
+  </si>
+  <si>
+    <t>Hiragana du (arm)</t>
+  </si>
+  <si>
+    <t>ﾉ</t>
+  </si>
+  <si>
+    <t>Halfwidth katakana no</t>
+  </si>
+  <si>
+    <t>ヘ</t>
+  </si>
+  <si>
+    <t>Katakana he</t>
+  </si>
+  <si>
+    <t>و</t>
+  </si>
+  <si>
+    <t>Arabic waw (decorative arm)</t>
+  </si>
+  <si>
+    <t>ఠ</t>
+  </si>
+  <si>
+    <t>Telugu ttha (eye)</t>
+  </si>
+  <si>
+    <t>ㅂ</t>
+  </si>
+  <si>
+    <t>Hangul pieup</t>
+  </si>
+  <si>
+    <t>丿</t>
+  </si>
+  <si>
+    <t>CJK slash radical (tail)</t>
+  </si>
+  <si>
+    <t>益</t>
+  </si>
+  <si>
+    <t>Kanji: benefit (angry mouth)</t>
   </si>
 </sst>
 </file>
@@ -12035,387 +12296,771 @@
       </c>
     </row>
     <row r="435" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A435" s="6"/>
-      <c r="B435" s="5"/>
-      <c r="C435" s="5"/>
+      <c r="A435" s="6" t="s">
+        <v>976</v>
+      </c>
+      <c r="B435" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C435" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D435" s="5"/>
-      <c r="E435" s="5"/>
+      <c r="E435" s="5" t="s">
+        <v>977</v>
+      </c>
       <c r="F435" s="5"/>
     </row>
     <row r="436" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A436" s="6"/>
-      <c r="B436" s="5"/>
-      <c r="C436" s="5"/>
+      <c r="A436" s="6" t="s">
+        <v>978</v>
+      </c>
+      <c r="B436" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C436" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D436" s="5"/>
-      <c r="E436" s="5"/>
+      <c r="E436" s="5" t="s">
+        <v>979</v>
+      </c>
       <c r="F436" s="5"/>
     </row>
     <row r="437" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A437" s="6"/>
-      <c r="B437" s="5"/>
-      <c r="C437" s="5"/>
+      <c r="A437" s="6" t="s">
+        <v>980</v>
+      </c>
+      <c r="B437" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C437" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D437" s="5"/>
-      <c r="E437" s="5"/>
+      <c r="E437" s="5" t="s">
+        <v>981</v>
+      </c>
       <c r="F437" s="5"/>
     </row>
     <row r="438" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A438" s="6"/>
-      <c r="B438" s="5"/>
-      <c r="C438" s="5"/>
+      <c r="A438" s="6" t="s">
+        <v>982</v>
+      </c>
+      <c r="B438" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C438" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D438" s="5"/>
-      <c r="E438" s="5"/>
+      <c r="E438" s="5" t="s">
+        <v>983</v>
+      </c>
       <c r="F438" s="5"/>
     </row>
     <row r="439" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A439" s="6"/>
-      <c r="B439" s="5"/>
-      <c r="C439" s="5"/>
+      <c r="A439" s="6" t="s">
+        <v>984</v>
+      </c>
+      <c r="B439" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C439" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D439" s="5"/>
-      <c r="E439" s="5"/>
+      <c r="E439" s="5" t="s">
+        <v>985</v>
+      </c>
       <c r="F439" s="5"/>
     </row>
     <row r="440" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A440" s="6"/>
-      <c r="B440" s="5"/>
-      <c r="C440" s="5"/>
+      <c r="A440" s="6" t="s">
+        <v>986</v>
+      </c>
+      <c r="B440" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C440" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D440" s="5"/>
-      <c r="E440" s="5"/>
+      <c r="E440" s="5" t="s">
+        <v>987</v>
+      </c>
       <c r="F440" s="5"/>
     </row>
     <row r="441" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A441" s="6"/>
-      <c r="B441" s="5"/>
-      <c r="C441" s="5"/>
+      <c r="A441" s="6" t="s">
+        <v>988</v>
+      </c>
+      <c r="B441" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C441" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D441" s="5"/>
-      <c r="E441" s="5"/>
+      <c r="E441" s="5" t="s">
+        <v>989</v>
+      </c>
       <c r="F441" s="5"/>
     </row>
     <row r="442" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A442" s="6"/>
-      <c r="B442" s="5"/>
-      <c r="C442" s="5"/>
+      <c r="A442" s="6" t="s">
+        <v>990</v>
+      </c>
+      <c r="B442" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C442" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D442" s="5"/>
-      <c r="E442" s="5"/>
+      <c r="E442" s="5" t="s">
+        <v>991</v>
+      </c>
       <c r="F442" s="5"/>
     </row>
     <row r="443" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A443" s="6"/>
-      <c r="B443" s="5"/>
-      <c r="C443" s="5"/>
+      <c r="A443" s="6" t="s">
+        <v>992</v>
+      </c>
+      <c r="B443" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C443" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D443" s="5"/>
-      <c r="E443" s="5"/>
+      <c r="E443" s="5" t="s">
+        <v>993</v>
+      </c>
       <c r="F443" s="5"/>
     </row>
     <row r="444" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A444" s="6"/>
-      <c r="B444" s="5"/>
-      <c r="C444" s="5"/>
+      <c r="A444" s="6" t="s">
+        <v>994</v>
+      </c>
+      <c r="B444" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C444" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D444" s="5"/>
-      <c r="E444" s="5"/>
+      <c r="E444" s="5" t="s">
+        <v>995</v>
+      </c>
       <c r="F444" s="5"/>
     </row>
     <row r="445" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A445" s="6"/>
-      <c r="B445" s="5"/>
-      <c r="C445" s="5"/>
+      <c r="A445" s="6" t="s">
+        <v>996</v>
+      </c>
+      <c r="B445" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C445" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D445" s="5"/>
-      <c r="E445" s="5"/>
+      <c r="E445" s="5" t="s">
+        <v>997</v>
+      </c>
       <c r="F445" s="5"/>
     </row>
     <row r="446" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A446" s="6"/>
-      <c r="B446" s="5"/>
-      <c r="C446" s="5"/>
+      <c r="A446" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B446" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C446" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D446" s="5"/>
-      <c r="E446" s="5"/>
+      <c r="E446" s="5" t="s">
+        <v>369</v>
+      </c>
       <c r="F446" s="5"/>
     </row>
     <row r="447" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A447" s="6"/>
-      <c r="B447" s="5"/>
-      <c r="C447" s="5"/>
+      <c r="A447" s="6" t="s">
+        <v>998</v>
+      </c>
+      <c r="B447" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C447" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D447" s="5"/>
-      <c r="E447" s="5"/>
+      <c r="E447" s="5" t="s">
+        <v>999</v>
+      </c>
       <c r="F447" s="5"/>
     </row>
     <row r="448" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A448" s="6"/>
-      <c r="B448" s="5"/>
-      <c r="C448" s="5"/>
+      <c r="A448" s="6" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B448" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C448" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D448" s="5"/>
-      <c r="E448" s="5"/>
+      <c r="E448" s="5" t="s">
+        <v>1001</v>
+      </c>
       <c r="F448" s="5"/>
     </row>
     <row r="449" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A449" s="6"/>
-      <c r="B449" s="5"/>
-      <c r="C449" s="5"/>
+      <c r="A449" s="6" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B449" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C449" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D449" s="5"/>
-      <c r="E449" s="5"/>
+      <c r="E449" s="5" t="s">
+        <v>1003</v>
+      </c>
       <c r="F449" s="5"/>
     </row>
     <row r="450" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A450" s="6"/>
-      <c r="B450" s="5"/>
-      <c r="C450" s="5"/>
+      <c r="A450" s="6" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B450" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C450" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D450" s="5"/>
-      <c r="E450" s="5"/>
+      <c r="E450" s="5" t="s">
+        <v>1005</v>
+      </c>
       <c r="F450" s="5"/>
     </row>
     <row r="451" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A451" s="6"/>
-      <c r="B451" s="5"/>
-      <c r="C451" s="5"/>
+      <c r="A451" s="6" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B451" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C451" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D451" s="5"/>
-      <c r="E451" s="5"/>
+      <c r="E451" s="5" t="s">
+        <v>1007</v>
+      </c>
       <c r="F451" s="5"/>
     </row>
     <row r="452" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A452" s="6"/>
-      <c r="B452" s="5"/>
-      <c r="C452" s="5"/>
+      <c r="A452" s="6" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B452" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C452" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D452" s="5"/>
-      <c r="E452" s="5"/>
+      <c r="E452" s="5" t="s">
+        <v>1009</v>
+      </c>
       <c r="F452" s="5"/>
     </row>
     <row r="453" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A453" s="6"/>
-      <c r="B453" s="5"/>
-      <c r="C453" s="5"/>
+      <c r="A453" s="6" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B453" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C453" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D453" s="5"/>
-      <c r="E453" s="5"/>
+      <c r="E453" s="5" t="s">
+        <v>1011</v>
+      </c>
       <c r="F453" s="5"/>
     </row>
     <row r="454" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A454" s="6"/>
-      <c r="B454" s="5"/>
-      <c r="C454" s="5"/>
+      <c r="A454" s="6" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B454" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C454" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D454" s="5"/>
-      <c r="E454" s="5"/>
+      <c r="E454" s="5" t="s">
+        <v>1013</v>
+      </c>
       <c r="F454" s="5"/>
     </row>
     <row r="455" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A455" s="6"/>
-      <c r="B455" s="5"/>
-      <c r="C455" s="5"/>
+      <c r="A455" s="6" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B455" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C455" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D455" s="5"/>
-      <c r="E455" s="5"/>
+      <c r="E455" s="5" t="s">
+        <v>1015</v>
+      </c>
       <c r="F455" s="5"/>
     </row>
     <row r="456" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A456" s="6"/>
-      <c r="B456" s="5"/>
-      <c r="C456" s="5"/>
+      <c r="A456" s="6" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B456" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C456" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D456" s="5"/>
-      <c r="E456" s="5"/>
+      <c r="E456" s="5" t="s">
+        <v>1017</v>
+      </c>
       <c r="F456" s="5"/>
     </row>
     <row r="457" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A457" s="6"/>
-      <c r="B457" s="5"/>
-      <c r="C457" s="5"/>
+      <c r="A457" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="B457" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C457" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D457" s="5"/>
-      <c r="E457" s="5"/>
+      <c r="E457" s="5" t="s">
+        <v>1018</v>
+      </c>
       <c r="F457" s="5"/>
     </row>
     <row r="458" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A458" s="6"/>
-      <c r="B458" s="5"/>
-      <c r="C458" s="5"/>
+      <c r="A458" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B458" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C458" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D458" s="5"/>
-      <c r="E458" s="5"/>
+      <c r="E458" s="5" t="s">
+        <v>1019</v>
+      </c>
       <c r="F458" s="5"/>
     </row>
     <row r="459" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A459" s="6"/>
-      <c r="B459" s="5"/>
-      <c r="C459" s="5"/>
+      <c r="A459" s="6" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B459" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C459" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D459" s="5"/>
-      <c r="E459" s="5"/>
+      <c r="E459" s="5" t="s">
+        <v>1021</v>
+      </c>
       <c r="F459" s="5"/>
     </row>
     <row r="460" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A460" s="6"/>
-      <c r="B460" s="5"/>
-      <c r="C460" s="5"/>
+      <c r="A460" s="6" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B460" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C460" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D460" s="5"/>
-      <c r="E460" s="5"/>
+      <c r="E460" s="5" t="s">
+        <v>1023</v>
+      </c>
       <c r="F460" s="5"/>
     </row>
     <row r="461" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A461" s="6"/>
-      <c r="B461" s="5"/>
-      <c r="C461" s="5"/>
+      <c r="A461" s="6" t="s">
+        <v>810</v>
+      </c>
+      <c r="B461" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C461" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D461" s="5"/>
-      <c r="E461" s="5"/>
+      <c r="E461" s="5" t="s">
+        <v>1024</v>
+      </c>
       <c r="F461" s="5"/>
     </row>
     <row r="462" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A462" s="6"/>
-      <c r="B462" s="5"/>
-      <c r="C462" s="5"/>
+      <c r="A462" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B462" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C462" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D462" s="5"/>
-      <c r="E462" s="5"/>
+      <c r="E462" s="5" t="s">
+        <v>370</v>
+      </c>
       <c r="F462" s="5"/>
     </row>
     <row r="463" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A463" s="6"/>
-      <c r="B463" s="5"/>
-      <c r="C463" s="5"/>
+      <c r="A463" s="6" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B463" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C463" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D463" s="5"/>
-      <c r="E463" s="5"/>
+      <c r="E463" s="5" t="s">
+        <v>1026</v>
+      </c>
       <c r="F463" s="5"/>
     </row>
     <row r="464" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A464" s="6"/>
-      <c r="B464" s="5"/>
-      <c r="C464" s="5"/>
+      <c r="A464" s="6" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B464" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C464" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D464" s="5"/>
-      <c r="E464" s="5"/>
+      <c r="E464" s="5" t="s">
+        <v>1028</v>
+      </c>
       <c r="F464" s="5"/>
     </row>
     <row r="465" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A465" s="6"/>
-      <c r="B465" s="5"/>
-      <c r="C465" s="5"/>
+      <c r="A465" s="6" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B465" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C465" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D465" s="5"/>
-      <c r="E465" s="5"/>
+      <c r="E465" s="5" t="s">
+        <v>1030</v>
+      </c>
       <c r="F465" s="5"/>
     </row>
     <row r="466" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A466" s="6"/>
-      <c r="B466" s="5"/>
-      <c r="C466" s="5"/>
+      <c r="A466" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B466" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C466" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D466" s="5"/>
-      <c r="E466" s="5"/>
+      <c r="E466" s="5" t="s">
+        <v>311</v>
+      </c>
       <c r="F466" s="5"/>
     </row>
     <row r="467" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A467" s="6"/>
-      <c r="B467" s="5"/>
-      <c r="C467" s="5"/>
+      <c r="A467" s="6" t="s">
+        <v>1031</v>
+      </c>
+      <c r="B467" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C467" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D467" s="5"/>
-      <c r="E467" s="5"/>
+      <c r="E467" s="5" t="s">
+        <v>1032</v>
+      </c>
       <c r="F467" s="5"/>
     </row>
     <row r="468" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A468" s="6"/>
-      <c r="B468" s="5"/>
-      <c r="C468" s="5"/>
+      <c r="A468" s="6" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B468" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C468" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D468" s="5"/>
-      <c r="E468" s="5"/>
+      <c r="E468" s="5" t="s">
+        <v>1034</v>
+      </c>
       <c r="F468" s="5"/>
     </row>
     <row r="469" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A469" s="6"/>
-      <c r="B469" s="5"/>
-      <c r="C469" s="5"/>
+      <c r="A469" s="6" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B469" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C469" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D469" s="5"/>
-      <c r="E469" s="5"/>
+      <c r="E469" s="5" t="s">
+        <v>1036</v>
+      </c>
       <c r="F469" s="5"/>
     </row>
     <row r="470" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A470" s="6"/>
-      <c r="B470" s="5"/>
-      <c r="C470" s="5"/>
+      <c r="A470" s="6" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B470" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C470" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D470" s="5"/>
-      <c r="E470" s="5"/>
+      <c r="E470" s="5" t="s">
+        <v>1038</v>
+      </c>
       <c r="F470" s="5"/>
     </row>
     <row r="471" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A471" s="6"/>
-      <c r="B471" s="5"/>
-      <c r="C471" s="5"/>
+      <c r="A471" s="6" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B471" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C471" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D471" s="5"/>
-      <c r="E471" s="5"/>
+      <c r="E471" s="5" t="s">
+        <v>1040</v>
+      </c>
       <c r="F471" s="5"/>
     </row>
     <row r="472" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A472" s="6"/>
-      <c r="B472" s="5"/>
-      <c r="C472" s="5"/>
+      <c r="A472" s="6" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B472" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C472" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D472" s="5"/>
-      <c r="E472" s="5"/>
+      <c r="E472" s="5" t="s">
+        <v>1042</v>
+      </c>
       <c r="F472" s="5"/>
     </row>
     <row r="473" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A473" s="6"/>
-      <c r="B473" s="5"/>
-      <c r="C473" s="5"/>
+      <c r="A473" s="6" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B473" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C473" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D473" s="5"/>
-      <c r="E473" s="5"/>
+      <c r="E473" s="5" t="s">
+        <v>1044</v>
+      </c>
       <c r="F473" s="5"/>
     </row>
     <row r="474" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A474" s="6"/>
-      <c r="B474" s="5"/>
-      <c r="C474" s="5"/>
+      <c r="A474" s="6" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B474" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C474" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D474" s="5"/>
-      <c r="E474" s="5"/>
+      <c r="E474" s="5" t="s">
+        <v>1046</v>
+      </c>
       <c r="F474" s="5"/>
     </row>
     <row r="475" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A475" s="6"/>
-      <c r="B475" s="5"/>
-      <c r="C475" s="5"/>
+      <c r="A475" s="6" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B475" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C475" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D475" s="5"/>
-      <c r="E475" s="5"/>
+      <c r="E475" s="5" t="s">
+        <v>1048</v>
+      </c>
       <c r="F475" s="5"/>
     </row>
     <row r="476" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A476" s="6"/>
-      <c r="B476" s="5"/>
-      <c r="C476" s="5"/>
+      <c r="A476" s="6" t="s">
+        <v>1049</v>
+      </c>
+      <c r="B476" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C476" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D476" s="5"/>
-      <c r="E476" s="5"/>
+      <c r="E476" s="5" t="s">
+        <v>1050</v>
+      </c>
       <c r="F476" s="5"/>
     </row>
     <row r="477" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A477" s="6"/>
-      <c r="B477" s="5"/>
-      <c r="C477" s="5"/>
+      <c r="A477" s="6" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B477" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C477" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D477" s="5"/>
-      <c r="E477" s="5"/>
+      <c r="E477" s="5" t="s">
+        <v>1052</v>
+      </c>
       <c r="F477" s="5"/>
     </row>
     <row r="478" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A478" s="6"/>
-      <c r="B478" s="5"/>
-      <c r="C478" s="5"/>
+      <c r="A478" s="6" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B478" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C478" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D478" s="5"/>
-      <c r="E478" s="5"/>
+      <c r="E478" s="5" t="s">
+        <v>1054</v>
+      </c>
       <c r="F478" s="5"/>
     </row>
     <row r="479" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A479" s="6"/>
-      <c r="B479" s="5"/>
-      <c r="C479" s="5"/>
+      <c r="A479" s="6" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B479" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C479" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D479" s="5"/>
-      <c r="E479" s="5"/>
+      <c r="E479" s="5" t="s">
+        <v>1056</v>
+      </c>
       <c r="F479" s="5"/>
     </row>
     <row r="480" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A480" s="6"/>
-      <c r="B480" s="5"/>
-      <c r="C480" s="5"/>
+      <c r="A480" s="6" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B480" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C480" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D480" s="5"/>
-      <c r="E480" s="5"/>
+      <c r="E480" s="5" t="s">
+        <v>1058</v>
+      </c>
       <c r="F480" s="5"/>
     </row>
     <row r="481" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A481" s="6"/>
-      <c r="B481" s="5"/>
-      <c r="C481" s="5"/>
+      <c r="A481" s="6" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B481" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C481" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D481" s="5"/>
-      <c r="E481" s="5"/>
+      <c r="E481" s="5" t="s">
+        <v>1060</v>
+      </c>
       <c r="F481" s="5"/>
     </row>
     <row r="482" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A482" s="6"/>
-      <c r="B482" s="5"/>
-      <c r="C482" s="5"/>
+      <c r="A482" s="6" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B482" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C482" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="D482" s="5"/>
-      <c r="E482" s="5"/>
+      <c r="E482" s="5" t="s">
+        <v>1062</v>
+      </c>
       <c r="F482" s="5"/>
     </row>
     <row r="483" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
@@ -32651,7 +33296,7 @@
       <c r="F3011" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F434" xr:uid="{E4EDB976-389A-4152-ACF3-6B6CAEFF159E}"/>
+  <autoFilter ref="A4:F482" xr:uid="{E4EDB976-389A-4152-ACF3-6B6CAEFF159E}"/>
   <conditionalFormatting sqref="C5:C3011">
     <cfRule type="cellIs" dxfId="2" priority="1" stopIfTrue="1" operator="equal">
       <formula>"Verified"</formula>

</xml_diff>